<commit_message>
agregando columna de unidad
</commit_message>
<xml_diff>
--- a/Computo y Presupuesto -Segovia Joaquin.xlsx
+++ b/Computo y Presupuesto -Segovia Joaquin.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andrea Fernandez\Documents\Pragma\presupuestador-obras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4426FE83-0E2E-4033-91FD-7230E4D1CD65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2678486F-705E-4CE0-A892-FA8F3A944E38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LISTA" sheetId="4" r:id="rId1"/>
@@ -3390,6 +3390,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="38" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="39" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="41" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="12" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3397,15 +3406,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="26" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="38" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="39" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="41" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3844,11 +3844,11 @@
         <v>21</v>
       </c>
       <c r="B5" s="59"/>
-      <c r="C5" s="342" t="s">
+      <c r="C5" s="339" t="s">
         <v>346</v>
       </c>
-      <c r="D5" s="343"/>
-      <c r="E5" s="344"/>
+      <c r="D5" s="340"/>
+      <c r="E5" s="341"/>
       <c r="F5" s="59"/>
     </row>
     <row r="6" spans="1:7" s="61" customFormat="1" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5444,13 +5444,13 @@
       <c r="A4" s="74"/>
     </row>
     <row r="5" spans="1:21" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="339" t="s">
+      <c r="B5" s="342" t="s">
         <v>127</v>
       </c>
-      <c r="C5" s="340"/>
-      <c r="D5" s="340"/>
-      <c r="E5" s="340"/>
-      <c r="F5" s="341"/>
+      <c r="C5" s="343"/>
+      <c r="D5" s="343"/>
+      <c r="E5" s="343"/>
+      <c r="F5" s="344"/>
       <c r="G5" s="78"/>
       <c r="U5" s="79">
         <v>333</v>

</xml_diff>